<commit_message>
updated the jenkins file
</commit_message>
<xml_diff>
--- a/src/test/java/resources/CreateUser_TestData.xlsx
+++ b/src/test/java/resources/CreateUser_TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jitesh\Desktop\BK_Selenium_git\FusionProject\src\test\java\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maagarwal\Downloads\FusionProject_Jenkins_Working\FusionProject\src\test\java\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ECAC428-BFEE-47ED-9507-6787DA5F1CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5F92F6-396D-43FA-85D0-F4B23E8E1F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,43 +36,85 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>demouser4</t>
-  </si>
-  <si>
-    <t>demouser4@test.com</t>
-  </si>
-  <si>
-    <t>Oracle@123</t>
-  </si>
-  <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>LastName</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>Confirm Password</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+  <si>
+    <t>hireReason</t>
+  </si>
+  <si>
+    <t>Hire to fill vacant position</t>
+  </si>
+  <si>
+    <t>legalEmployerField</t>
+  </si>
+  <si>
+    <t>IT CONVERGENCE PROFESSIONAL SERVICES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>lastNameField</t>
+  </si>
+  <si>
+    <t>firstNameField</t>
+  </si>
+  <si>
+    <t>addressLine1</t>
+  </si>
+  <si>
+    <t>ITC Testing Center</t>
+  </si>
+  <si>
+    <t>cityField</t>
+  </si>
+  <si>
+    <t>Hyderabad</t>
+  </si>
+  <si>
+    <t>addressLine2</t>
+  </si>
+  <si>
+    <t>DLF Cyber City</t>
+  </si>
+  <si>
+    <t>pinCodeField</t>
+  </si>
+  <si>
+    <t>businessUnitField</t>
+  </si>
+  <si>
+    <t>IT Convergence India - Hyderabad</t>
+  </si>
+  <si>
+    <t>500081</t>
+  </si>
+  <si>
+    <t>assignment</t>
+  </si>
+  <si>
+    <t>manager</t>
+  </si>
+  <si>
+    <t>timecardvalue</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Kalsi, Sharan</t>
+  </si>
+  <si>
+    <t>dummy222</t>
+  </si>
+  <si>
+    <t>290222</t>
+  </si>
+  <si>
+    <t>test222</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -81,27 +123,25 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -113,17 +153,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -402,63 +442,112 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.81640625" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.26953125" customWidth="1"/>
+    <col min="11" max="11" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="2">
-        <v>9876543210</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>3</v>
-      </c>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{B26F3378-980D-4454-BD77-A9BF497BB7CB}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{35ADBA0F-7C3D-4871-B37C-2933C443D2FC}"/>
-    <hyperlink ref="F2" r:id="rId3" xr:uid="{37A0A84E-5DD5-4B06-98BF-DD09AAF7ED04}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>